<commit_message>
New Clean order changes
</commit_message>
<xml_diff>
--- a/Data Files/OTM Test Data/Demo Bulk IDs.xlsx
+++ b/Data Files/OTM Test Data/Demo Bulk IDs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlueLinx_Automation_Master\Data Files\OTM Test Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PrajyotDabhade\Documents\BlueLinx_Automation_Master\Data Files\OTM Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7857C3D2-8786-4D28-AEBA-B2903158947C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8B134D-1CFF-444F-BF3E-26D80975BFA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{3033C71C-91B3-45AA-8870-5371DAB13ABE}"/>
   </bookViews>
@@ -25,24 +25,30 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>BULK IDs</t>
   </si>
   <si>
+    <t>20250902-0004</t>
+  </si>
+  <si>
     <t>20250902-0002</t>
   </si>
   <si>
+    <t>Status</t>
+  </si>
+  <si>
     <t>SECURE RESOURCES_WITHDRAWN</t>
   </si>
   <si>
     <t>SECURE RESOURCES_ACCEPTED</t>
   </si>
   <si>
-    <t>Current Status</t>
-  </si>
-  <si>
-    <t>20250903-0009</t>
+    <t>20250902-0008</t>
+  </si>
+  <si>
+    <t>SECURE RESOURCES_NOT STARTED</t>
   </si>
 </sst>
 </file>
@@ -409,12 +415,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6F13729-7653-44B7-8A16-E2DDDD80648E}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="16.08984375" customWidth="1"/>
     <col min="2" max="2" width="33.26953125" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -422,23 +427,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>2</v>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean up bulk id
</commit_message>
<xml_diff>
--- a/Data Files/OTM Test Data/Demo Bulk IDs.xlsx
+++ b/Data Files/OTM Test Data/Demo Bulk IDs.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PrajyotDabhade\Documents\BlueLinx_Automation_Master\Data Files\OTM Test Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\BlueLinx_Automation_Master\Data Files\OTM Test Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9C8B134D-1CFF-444F-BF3E-26D80975BFA4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{249FE258-C1A7-4A1A-AD81-876F888D47A5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6810" xr2:uid="{3033C71C-91B3-45AA-8870-5371DAB13ABE}"/>
   </bookViews>
@@ -25,30 +25,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>BULK IDs</t>
   </si>
   <si>
-    <t>20250902-0004</t>
+    <t>Captured Current Status</t>
   </si>
   <si>
-    <t>20250902-0002</t>
+    <t>Status After Execution</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
-    <t>SECURE RESOURCES_WITHDRAWN</t>
-  </si>
-  <si>
-    <t>SECURE RESOURCES_ACCEPTED</t>
-  </si>
-  <si>
-    <t>20250902-0008</t>
-  </si>
-  <si>
-    <t>SECURE RESOURCES_NOT STARTED</t>
+    <t>20250904-0002</t>
   </si>
 </sst>
 </file>
@@ -415,43 +403,28 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B6F13729-7653-44B7-8A16-E2DDDD80648E}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.08984375" customWidth="1"/>
-    <col min="2" max="2" width="33.26953125" customWidth="1"/>
+    <col min="1" max="1" width="16.08984375" customWidth="1" collapsed="1"/>
+    <col min="2" max="2" width="33.26953125" customWidth="1" collapsed="1"/>
+    <col min="3" max="3" width="26.453125" customWidth="1" collapsed="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>